<commit_message>
Phase B: complete n=20 (30/30 instances) and full analysis
- runs_full.csv: 540 runs (n=12,16,20 x 30 instances x 6 methods), same seeds as original run
- analysis_full.txt / phaseB_summary.xlsx: medians, Wilcoxon, A12, win/tie/loss
- n=20 median pairwise coverage: greedy 54.5%, GA 53.9%, SA 53.1%, QAOA 52.3%, random 47.1%

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122GSt9Zq6fddTq7qHbYi5D
</commit_message>
<xml_diff>
--- a/phaseB_qubo_scenario_selection/results/phaseB_summary.xlsx
+++ b/phaseB_qubo_scenario_selection/results/phaseB_summary.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="434">
   <si>
     <t>n</t>
   </si>
@@ -1117,6 +1117,207 @@
   </si>
   <si>
     <t>4 7 10 11 16</t>
+  </si>
+  <si>
+    <t>0 1 2 3 8</t>
+  </si>
+  <si>
+    <t>0 1 10 14 15</t>
+  </si>
+  <si>
+    <t>2 8 10 11 18</t>
+  </si>
+  <si>
+    <t>8 10 11 17 18</t>
+  </si>
+  <si>
+    <t>1 4 8 10 14</t>
+  </si>
+  <si>
+    <t>0 1 3 8 17</t>
+  </si>
+  <si>
+    <t>6 9 11 12 13</t>
+  </si>
+  <si>
+    <t>2 10 11 12 13</t>
+  </si>
+  <si>
+    <t>10 11 12 13 16</t>
+  </si>
+  <si>
+    <t>6 7 8 9 11</t>
+  </si>
+  <si>
+    <t>1 2 3 4 11</t>
+  </si>
+  <si>
+    <t>1 2 11 14 17</t>
+  </si>
+  <si>
+    <t>2 11 14 16 17</t>
+  </si>
+  <si>
+    <t>1 2 10 11 14</t>
+  </si>
+  <si>
+    <t>4 11 16 18 19</t>
+  </si>
+  <si>
+    <t>1 2 4 5 9</t>
+  </si>
+  <si>
+    <t>4 5 9 10 18</t>
+  </si>
+  <si>
+    <t>5 8 9 10 18</t>
+  </si>
+  <si>
+    <t>5 8 14 16 18</t>
+  </si>
+  <si>
+    <t>4 8 12 14 16</t>
+  </si>
+  <si>
+    <t>0 1 3 10 13</t>
+  </si>
+  <si>
+    <t>5 7 10 11 19</t>
+  </si>
+  <si>
+    <t>2 11 13 15 19</t>
+  </si>
+  <si>
+    <t>2 3 11 13 19</t>
+  </si>
+  <si>
+    <t>3 5 10 13 17</t>
+  </si>
+  <si>
+    <t>1 3 7 16 18</t>
+  </si>
+  <si>
+    <t>7 9 14 16 18</t>
+  </si>
+  <si>
+    <t>7 8 9 16 18</t>
+  </si>
+  <si>
+    <t>5 7 9 16 18</t>
+  </si>
+  <si>
+    <t>4 6 8 14 17</t>
+  </si>
+  <si>
+    <t>0 2 4 6 13</t>
+  </si>
+  <si>
+    <t>2 6 9 13 18</t>
+  </si>
+  <si>
+    <t>0 3 6 9 13</t>
+  </si>
+  <si>
+    <t>0 2 4 6 9</t>
+  </si>
+  <si>
+    <t>0 7 8 11 16</t>
+  </si>
+  <si>
+    <t>1 5 15 16 17</t>
+  </si>
+  <si>
+    <t>5 15 16 17 19</t>
+  </si>
+  <si>
+    <t>5 12 15 16 17</t>
+  </si>
+  <si>
+    <t>5 12 15 16 19</t>
+  </si>
+  <si>
+    <t>1 2 3 9 16</t>
+  </si>
+  <si>
+    <t>0 1 4 5 16</t>
+  </si>
+  <si>
+    <t>0 3 11 16 19</t>
+  </si>
+  <si>
+    <t>0 2 3 4 19</t>
+  </si>
+  <si>
+    <t>0 3 6 8 19</t>
+  </si>
+  <si>
+    <t>5 9 10 13 15</t>
+  </si>
+  <si>
+    <t>0 6 9 10 16</t>
+  </si>
+  <si>
+    <t>2 4 12 16 18</t>
+  </si>
+  <si>
+    <t>2 4 5 12 16</t>
+  </si>
+  <si>
+    <t>2 12 16 18 19</t>
+  </si>
+  <si>
+    <t>1 4 8 16 17</t>
+  </si>
+  <si>
+    <t>0 1 2 10 15</t>
+  </si>
+  <si>
+    <t>2 6 9 14 15</t>
+  </si>
+  <si>
+    <t>0 2 4 9 15</t>
+  </si>
+  <si>
+    <t>2 4 6 9 14</t>
+  </si>
+  <si>
+    <t>6 7 12 14 18</t>
+  </si>
+  <si>
+    <t>0 2 4 7 8</t>
+  </si>
+  <si>
+    <t>1 7 14 15 19</t>
+  </si>
+  <si>
+    <t>1 7 14 15 16</t>
+  </si>
+  <si>
+    <t>5 7 15 17 18</t>
+  </si>
+  <si>
+    <t>2 8 10 14 18</t>
+  </si>
+  <si>
+    <t>0 1 2 7 11</t>
+  </si>
+  <si>
+    <t>1 2 8 11 18</t>
+  </si>
+  <si>
+    <t>1 8 11 14 18</t>
+  </si>
+  <si>
+    <t>1 3 8 16 18</t>
+  </si>
+  <si>
+    <t>3 10 15 18 19</t>
+  </si>
+  <si>
+    <t>1 2 6 7 10</t>
+  </si>
+  <si>
+    <t>2 7 10 15 18</t>
   </si>
 </sst>
 </file>
@@ -2460,22 +2661,22 @@
         <v>25</v>
       </c>
       <c r="C14">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D14">
-        <v>0.4646401985111662</v>
+        <v>0.4710972451141982</v>
       </c>
       <c r="E14">
-        <v>0.4571964841604101</v>
+        <v>0.4574300354749704</v>
       </c>
       <c r="F14">
-        <v>0.4815094662408759</v>
+        <v>0.4916582406471183</v>
       </c>
       <c r="G14">
         <v>0.8461538461538461</v>
       </c>
       <c r="H14">
-        <v>0.75</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="I14">
         <v>0.9230769230769232</v>
@@ -2511,10 +2712,10 @@
         <v>12.36671784755822</v>
       </c>
       <c r="T14">
-        <v>9.134005289044921</v>
+        <v>9.260830433341539</v>
       </c>
       <c r="U14">
-        <v>14.11069647635134</v>
+        <v>14.14881559839239</v>
       </c>
       <c r="V14">
         <v>0.0002</v>
@@ -2537,22 +2738,22 @@
         <v>26</v>
       </c>
       <c r="C15">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D15">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="E15">
-        <v>0.5342220053951673</v>
+        <v>0.5350917169875812</v>
       </c>
       <c r="F15">
-        <v>0.548828125</v>
+        <v>0.5617055084745762</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15">
-        <v>0.9230769230769232</v>
+        <v>0.9423076923076924</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -2585,22 +2786,22 @@
         <v>1</v>
       </c>
       <c r="S15">
-        <v>5.345167478048893</v>
+        <v>4.581379864167843</v>
       </c>
       <c r="T15">
-        <v>3.599452852242109</v>
+        <v>3.39874720108179</v>
       </c>
       <c r="U15">
-        <v>6.285662491673577</v>
+        <v>6.14236274458159</v>
       </c>
       <c r="V15">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="W15">
         <v>0.0002</v>
       </c>
       <c r="X15">
-        <v>0.0003</v>
+        <v>0.000375</v>
       </c>
       <c r="Y15">
         <v>0</v>
@@ -2614,16 +2815,16 @@
         <v>27</v>
       </c>
       <c r="C16">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D16">
         <v>0.5384615384615384</v>
       </c>
       <c r="E16">
-        <v>0.5310132575757576</v>
+        <v>0.5257395313100269</v>
       </c>
       <c r="F16">
-        <v>0.54615218996063</v>
+        <v>0.5536125242248062</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -2665,19 +2866,19 @@
         <v>5.887396014259139E-06</v>
       </c>
       <c r="T16">
-        <v>-5.368956095708199E-06</v>
+        <v>-1.242372869114661E-05</v>
       </c>
       <c r="U16">
-        <v>2.676098020515383E-05</v>
+        <v>2.509494089508735E-05</v>
       </c>
       <c r="V16">
-        <v>0.26185</v>
+        <v>0.30485</v>
       </c>
       <c r="W16">
-        <v>0.25475</v>
+        <v>0.261625</v>
       </c>
       <c r="X16">
-        <v>0.29335</v>
+        <v>0.3325</v>
       </c>
       <c r="Y16">
         <v>1</v>
@@ -2691,19 +2892,19 @@
         <v>28</v>
       </c>
       <c r="C17">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D17">
-        <v>0.5323019086176981</v>
+        <v>0.5310096153846153</v>
       </c>
       <c r="E17">
-        <v>0.518875020894857</v>
+        <v>0.5184571237532736</v>
       </c>
       <c r="F17">
-        <v>0.5407381186899778</v>
+        <v>0.5456524332061069</v>
       </c>
       <c r="G17">
-        <v>0.9615384615384617</v>
+        <v>0.9230769230769232</v>
       </c>
       <c r="H17">
         <v>0.9230769230769232</v>
@@ -2739,25 +2940,25 @@
         <v>1</v>
       </c>
       <c r="S17">
-        <v>1.344056895293079</v>
+        <v>1.325613565619278</v>
       </c>
       <c r="T17">
-        <v>0.9667250906335313</v>
+        <v>0.9199266523271773</v>
       </c>
       <c r="U17">
-        <v>1.620535025277491</v>
+        <v>1.706258613499955</v>
       </c>
       <c r="V17">
-        <v>0.05</v>
+        <v>0.0614</v>
       </c>
       <c r="W17">
-        <v>0.048625</v>
+        <v>0.04995</v>
       </c>
       <c r="X17">
-        <v>0.050825</v>
+        <v>0.083825</v>
       </c>
       <c r="Y17">
-        <v>0.0625</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -2768,16 +2969,16 @@
         <v>29</v>
       </c>
       <c r="C18">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D18">
-        <v>0.5248972401644157</v>
+        <v>0.5234432234432235</v>
       </c>
       <c r="E18">
-        <v>0.5168349706382745</v>
+        <v>0.5151002798507462</v>
       </c>
       <c r="F18">
-        <v>0.5329144786196549</v>
+        <v>0.5320060483870968</v>
       </c>
       <c r="G18">
         <v>0.9230769230769232</v>
@@ -2816,22 +3017,22 @@
         <v>1</v>
       </c>
       <c r="S18">
-        <v>2.817435447446485</v>
+        <v>2.655214934127343</v>
       </c>
       <c r="T18">
-        <v>2.154835061286661</v>
+        <v>1.861500388242945</v>
       </c>
       <c r="U18">
-        <v>3.424523097976561</v>
+        <v>3.316857015748639</v>
       </c>
       <c r="V18">
-        <v>180.3522</v>
+        <v>184.7845</v>
       </c>
       <c r="W18">
-        <v>179.332975</v>
+        <v>180.3457</v>
       </c>
       <c r="X18">
-        <v>182.207025</v>
+        <v>205.557575</v>
       </c>
       <c r="Y18">
         <v>0</v>
@@ -2845,16 +3046,16 @@
         <v>30</v>
       </c>
       <c r="C19">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D19">
         <v>0.5384615384615384</v>
       </c>
       <c r="E19">
-        <v>0.5310132575757576</v>
+        <v>0.5257395313100269</v>
       </c>
       <c r="F19">
-        <v>0.54615218996063</v>
+        <v>0.5536125242248062</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -2896,19 +3097,19 @@
         <v>5.887396014259139E-06</v>
       </c>
       <c r="T19">
-        <v>-5.368956095708199E-06</v>
+        <v>-1.242372869114661E-05</v>
       </c>
       <c r="U19">
-        <v>2.676098020515383E-05</v>
+        <v>2.509494089508735E-05</v>
       </c>
       <c r="V19">
-        <v>0.2516</v>
+        <v>0.2709</v>
       </c>
       <c r="W19">
-        <v>0.2388</v>
+        <v>0.24665</v>
       </c>
       <c r="X19">
-        <v>0.274225</v>
+        <v>0.29055</v>
       </c>
       <c r="Y19">
         <v>1</v>
@@ -3607,16 +3808,16 @@
         <v>39</v>
       </c>
       <c r="D22">
-        <v>0.4646401985111662</v>
+        <v>0.4710972451141982</v>
       </c>
       <c r="E22">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="F22">
-        <v>3.0517578125E-05</v>
+        <v>1.862645149230957E-09</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -3625,7 +3826,7 @@
         <v>0</v>
       </c>
       <c r="J22">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -3645,19 +3846,19 @@
         <v>1</v>
       </c>
       <c r="F23">
-        <v>0.001434633213931006</v>
+        <v>1.187575691792057E-05</v>
       </c>
       <c r="G23">
-        <v>0.08984375</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23">
         <v>3</v>
       </c>
       <c r="J23">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -3674,22 +3875,22 @@
         <v>0.5384615384615384</v>
       </c>
       <c r="E24">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="F24">
-        <v>0.09249147011262995</v>
+        <v>0.01759382050056426</v>
       </c>
       <c r="G24">
-        <v>0.4140625</v>
+        <v>0.38</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J24">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -3709,19 +3910,19 @@
         <v>1</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>0.8083651559145103</v>
       </c>
       <c r="G25">
-        <v>0.5</v>
+        <v>0.4561111111111111</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I25">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3735,25 +3936,25 @@
         <v>39</v>
       </c>
       <c r="D26">
-        <v>0.5323019086176981</v>
+        <v>0.5310096153846153</v>
       </c>
       <c r="E26">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="F26">
-        <v>0.003239921272238346</v>
+        <v>0.0002271386087118297</v>
       </c>
       <c r="G26">
-        <v>0.298828125</v>
+        <v>0.2961111111111111</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J26">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3767,25 +3968,25 @@
         <v>40</v>
       </c>
       <c r="D27">
-        <v>0.9615384615384617</v>
+        <v>0.9230769230769232</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27">
-        <v>0.09558070454562941</v>
+        <v>0.02256172310705745</v>
       </c>
       <c r="G27">
-        <v>0.396484375</v>
+        <v>0.3366666666666667</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J27">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -3799,25 +4000,25 @@
         <v>39</v>
       </c>
       <c r="D28">
-        <v>0.5248972401644157</v>
+        <v>0.5234432234432235</v>
       </c>
       <c r="E28">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="F28">
-        <v>0.0009815397525216685</v>
+        <v>9.338596171049022E-06</v>
       </c>
       <c r="G28">
-        <v>0.203125</v>
+        <v>0.1994444444444445</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J28">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -3837,19 +4038,19 @@
         <v>1</v>
       </c>
       <c r="F29">
-        <v>0.02585758046344292</v>
+        <v>0.008021790441065765</v>
       </c>
       <c r="G29">
-        <v>0.283203125</v>
+        <v>0.2955555555555556</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J29">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -3866,22 +4067,22 @@
         <v>0.5384615384615384</v>
       </c>
       <c r="E30">
-        <v>0.5411536567347943</v>
+        <v>0.5447304663840097</v>
       </c>
       <c r="F30">
-        <v>0.1281901743451078</v>
+        <v>0.02452044582672338</v>
       </c>
       <c r="G30">
-        <v>0.416015625</v>
+        <v>0.3838888888888889</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J30">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -3901,19 +4102,19 @@
         <v>1</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>0.8083651559145103</v>
       </c>
       <c r="G31">
-        <v>0.5</v>
+        <v>0.4561111111111111</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I31">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J31">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3923,7 +4124,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q457"/>
+  <dimension ref="A1:Q541"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -25867,6 +26068,4038 @@
         <v>366</v>
       </c>
     </row>
+    <row r="458" spans="1:17">
+      <c r="A458">
+        <v>20</v>
+      </c>
+      <c r="B458">
+        <v>5</v>
+      </c>
+      <c r="C458">
+        <v>20280943</v>
+      </c>
+      <c r="D458" t="s">
+        <v>25</v>
+      </c>
+      <c r="E458">
+        <v>0.0002</v>
+      </c>
+      <c r="F458">
+        <v>-28.55375457875459</v>
+      </c>
+      <c r="G458">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H458">
+        <v>12.99917832818221</v>
+      </c>
+      <c r="I458">
+        <v>5</v>
+      </c>
+      <c r="J458">
+        <v>1</v>
+      </c>
+      <c r="K458">
+        <v>0.4841269841269841</v>
+      </c>
+      <c r="L458">
+        <v>0.875</v>
+      </c>
+      <c r="M458">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N458">
+        <v>1</v>
+      </c>
+      <c r="Q458" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="459" spans="1:17">
+      <c r="A459">
+        <v>20</v>
+      </c>
+      <c r="B459">
+        <v>5</v>
+      </c>
+      <c r="C459">
+        <v>20280943</v>
+      </c>
+      <c r="D459" t="s">
+        <v>26</v>
+      </c>
+      <c r="E459">
+        <v>0.0003</v>
+      </c>
+      <c r="F459">
+        <v>-35.20018315018308</v>
+      </c>
+      <c r="G459">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H459">
+        <v>6.352749756753724</v>
+      </c>
+      <c r="I459">
+        <v>5</v>
+      </c>
+      <c r="J459">
+        <v>1</v>
+      </c>
+      <c r="K459">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="L459">
+        <v>1</v>
+      </c>
+      <c r="M459">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N459">
+        <v>1</v>
+      </c>
+      <c r="Q459" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="460" spans="1:17">
+      <c r="A460">
+        <v>20</v>
+      </c>
+      <c r="B460">
+        <v>5</v>
+      </c>
+      <c r="C460">
+        <v>20280943</v>
+      </c>
+      <c r="D460" t="s">
+        <v>30</v>
+      </c>
+      <c r="E460">
+        <v>0.2915</v>
+      </c>
+      <c r="F460">
+        <v>-41.55293040293032</v>
+      </c>
+      <c r="G460">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H460">
+        <v>2.504006488379673E-06</v>
+      </c>
+      <c r="I460">
+        <v>5</v>
+      </c>
+      <c r="J460">
+        <v>1</v>
+      </c>
+      <c r="K460">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="L460">
+        <v>1</v>
+      </c>
+      <c r="M460">
+        <v>1</v>
+      </c>
+      <c r="N460">
+        <v>1</v>
+      </c>
+      <c r="Q460" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="461" spans="1:17">
+      <c r="A461">
+        <v>20</v>
+      </c>
+      <c r="B461">
+        <v>5</v>
+      </c>
+      <c r="C461">
+        <v>20280943</v>
+      </c>
+      <c r="D461" t="s">
+        <v>28</v>
+      </c>
+      <c r="E461">
+        <v>2.5484</v>
+      </c>
+      <c r="F461">
+        <v>-39.44816849816834</v>
+      </c>
+      <c r="G461">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H461">
+        <v>2.10476440876846</v>
+      </c>
+      <c r="I461">
+        <v>5</v>
+      </c>
+      <c r="J461">
+        <v>1</v>
+      </c>
+      <c r="K461">
+        <v>0.5634920634920635</v>
+      </c>
+      <c r="L461">
+        <v>1</v>
+      </c>
+      <c r="M461">
+        <v>1</v>
+      </c>
+      <c r="N461">
+        <v>1</v>
+      </c>
+      <c r="Q461" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="462" spans="1:17">
+      <c r="A462">
+        <v>20</v>
+      </c>
+      <c r="B462">
+        <v>5</v>
+      </c>
+      <c r="C462">
+        <v>20280943</v>
+      </c>
+      <c r="D462" t="s">
+        <v>27</v>
+      </c>
+      <c r="E462">
+        <v>0.5204</v>
+      </c>
+      <c r="F462">
+        <v>-41.55293040293032</v>
+      </c>
+      <c r="G462">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H462">
+        <v>2.504006488379673E-06</v>
+      </c>
+      <c r="I462">
+        <v>5</v>
+      </c>
+      <c r="J462">
+        <v>1</v>
+      </c>
+      <c r="K462">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="L462">
+        <v>1</v>
+      </c>
+      <c r="M462">
+        <v>1</v>
+      </c>
+      <c r="N462">
+        <v>1</v>
+      </c>
+      <c r="Q462" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="463" spans="1:17">
+      <c r="A463">
+        <v>20</v>
+      </c>
+      <c r="B463">
+        <v>5</v>
+      </c>
+      <c r="C463">
+        <v>20280943</v>
+      </c>
+      <c r="D463" t="s">
+        <v>29</v>
+      </c>
+      <c r="E463">
+        <v>203.4869</v>
+      </c>
+      <c r="F463">
+        <v>-37.75412087912082</v>
+      </c>
+      <c r="G463">
+        <v>-41.5529329069368</v>
+      </c>
+      <c r="H463">
+        <v>3.798812027815984</v>
+      </c>
+      <c r="I463">
+        <v>5</v>
+      </c>
+      <c r="J463">
+        <v>1</v>
+      </c>
+      <c r="K463">
+        <v>0.5238095238095238</v>
+      </c>
+      <c r="L463">
+        <v>1</v>
+      </c>
+      <c r="M463">
+        <v>1</v>
+      </c>
+      <c r="N463">
+        <v>1</v>
+      </c>
+      <c r="O463">
+        <v>1.815134734391893E-05</v>
+      </c>
+      <c r="P463">
+        <v>450</v>
+      </c>
+      <c r="Q463" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="464" spans="1:17">
+      <c r="A464">
+        <v>20</v>
+      </c>
+      <c r="B464">
+        <v>5</v>
+      </c>
+      <c r="C464">
+        <v>20280944</v>
+      </c>
+      <c r="D464" t="s">
+        <v>25</v>
+      </c>
+      <c r="E464">
+        <v>0.0002</v>
+      </c>
+      <c r="F464">
+        <v>-27.35370046620051</v>
+      </c>
+      <c r="G464">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H464">
+        <v>9.821817436307128</v>
+      </c>
+      <c r="I464">
+        <v>5</v>
+      </c>
+      <c r="J464">
+        <v>1</v>
+      </c>
+      <c r="K464">
+        <v>0.4841269841269841</v>
+      </c>
+      <c r="L464">
+        <v>1</v>
+      </c>
+      <c r="M464">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N464">
+        <v>1</v>
+      </c>
+      <c r="Q464" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="465" spans="1:17">
+      <c r="A465">
+        <v>20</v>
+      </c>
+      <c r="B465">
+        <v>5</v>
+      </c>
+      <c r="C465">
+        <v>20280944</v>
+      </c>
+      <c r="D465" t="s">
+        <v>26</v>
+      </c>
+      <c r="E465">
+        <v>0.0003</v>
+      </c>
+      <c r="F465">
+        <v>-32.613956876457</v>
+      </c>
+      <c r="G465">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H465">
+        <v>4.56156102605064</v>
+      </c>
+      <c r="I465">
+        <v>5</v>
+      </c>
+      <c r="J465">
+        <v>1</v>
+      </c>
+      <c r="K465">
+        <v>0.5634920634920635</v>
+      </c>
+      <c r="L465">
+        <v>1</v>
+      </c>
+      <c r="M465">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N465">
+        <v>1</v>
+      </c>
+      <c r="Q465" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="466" spans="1:17">
+      <c r="A466">
+        <v>20</v>
+      </c>
+      <c r="B466">
+        <v>5</v>
+      </c>
+      <c r="C466">
+        <v>20280944</v>
+      </c>
+      <c r="D466" t="s">
+        <v>30</v>
+      </c>
+      <c r="E466">
+        <v>0.298</v>
+      </c>
+      <c r="F466">
+        <v>-37.17549533799547</v>
+      </c>
+      <c r="G466">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H466">
+        <v>2.25645121645357E-05</v>
+      </c>
+      <c r="I466">
+        <v>5</v>
+      </c>
+      <c r="J466">
+        <v>1</v>
+      </c>
+      <c r="K466">
+        <v>0.5634920634920635</v>
+      </c>
+      <c r="L466">
+        <v>1</v>
+      </c>
+      <c r="M466">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N466">
+        <v>1</v>
+      </c>
+      <c r="Q466" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="467" spans="1:17">
+      <c r="A467">
+        <v>20</v>
+      </c>
+      <c r="B467">
+        <v>5</v>
+      </c>
+      <c r="C467">
+        <v>20280944</v>
+      </c>
+      <c r="D467" t="s">
+        <v>28</v>
+      </c>
+      <c r="E467">
+        <v>0.0827</v>
+      </c>
+      <c r="F467">
+        <v>-34.65786713286718</v>
+      </c>
+      <c r="G467">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H467">
+        <v>2.517650769640454</v>
+      </c>
+      <c r="I467">
+        <v>5</v>
+      </c>
+      <c r="J467">
+        <v>1</v>
+      </c>
+      <c r="K467">
+        <v>0.5158730158730159</v>
+      </c>
+      <c r="L467">
+        <v>1</v>
+      </c>
+      <c r="M467">
+        <v>1</v>
+      </c>
+      <c r="N467">
+        <v>1</v>
+      </c>
+      <c r="Q467" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="468" spans="1:17">
+      <c r="A468">
+        <v>20</v>
+      </c>
+      <c r="B468">
+        <v>5</v>
+      </c>
+      <c r="C468">
+        <v>20280944</v>
+      </c>
+      <c r="D468" t="s">
+        <v>27</v>
+      </c>
+      <c r="E468">
+        <v>0.3651</v>
+      </c>
+      <c r="F468">
+        <v>-37.17549533799547</v>
+      </c>
+      <c r="G468">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H468">
+        <v>2.25645121645357E-05</v>
+      </c>
+      <c r="I468">
+        <v>5</v>
+      </c>
+      <c r="J468">
+        <v>1</v>
+      </c>
+      <c r="K468">
+        <v>0.5634920634920635</v>
+      </c>
+      <c r="L468">
+        <v>1</v>
+      </c>
+      <c r="M468">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N468">
+        <v>1</v>
+      </c>
+      <c r="Q468" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="469" spans="1:17">
+      <c r="A469">
+        <v>20</v>
+      </c>
+      <c r="B469">
+        <v>5</v>
+      </c>
+      <c r="C469">
+        <v>20280944</v>
+      </c>
+      <c r="D469" t="s">
+        <v>29</v>
+      </c>
+      <c r="E469">
+        <v>207.181</v>
+      </c>
+      <c r="F469">
+        <v>-35.40087412587422</v>
+      </c>
+      <c r="G469">
+        <v>-37.17551790250764</v>
+      </c>
+      <c r="H469">
+        <v>1.774643776633411</v>
+      </c>
+      <c r="I469">
+        <v>5</v>
+      </c>
+      <c r="J469">
+        <v>1</v>
+      </c>
+      <c r="K469">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="L469">
+        <v>1</v>
+      </c>
+      <c r="M469">
+        <v>1</v>
+      </c>
+      <c r="N469">
+        <v>1</v>
+      </c>
+      <c r="O469">
+        <v>1.758874183412847E-05</v>
+      </c>
+      <c r="P469">
+        <v>450</v>
+      </c>
+      <c r="Q469" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="470" spans="1:17">
+      <c r="A470">
+        <v>20</v>
+      </c>
+      <c r="B470">
+        <v>5</v>
+      </c>
+      <c r="C470">
+        <v>20280945</v>
+      </c>
+      <c r="D470" t="s">
+        <v>25</v>
+      </c>
+      <c r="E470">
+        <v>0.0002</v>
+      </c>
+      <c r="F470">
+        <v>-27.51036463536479</v>
+      </c>
+      <c r="G470">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H470">
+        <v>10.6262778969076</v>
+      </c>
+      <c r="I470">
+        <v>5</v>
+      </c>
+      <c r="J470">
+        <v>1</v>
+      </c>
+      <c r="K470">
+        <v>0.4960629921259842</v>
+      </c>
+      <c r="L470">
+        <v>1</v>
+      </c>
+      <c r="M470">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N470">
+        <v>1</v>
+      </c>
+      <c r="Q470" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="471" spans="1:17">
+      <c r="A471">
+        <v>20</v>
+      </c>
+      <c r="B471">
+        <v>5</v>
+      </c>
+      <c r="C471">
+        <v>20280945</v>
+      </c>
+      <c r="D471" t="s">
+        <v>26</v>
+      </c>
+      <c r="E471">
+        <v>0.0003</v>
+      </c>
+      <c r="F471">
+        <v>-35.71370712620717</v>
+      </c>
+      <c r="G471">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H471">
+        <v>2.422935406065221</v>
+      </c>
+      <c r="I471">
+        <v>5</v>
+      </c>
+      <c r="J471">
+        <v>1</v>
+      </c>
+      <c r="K471">
+        <v>0.5669291338582677</v>
+      </c>
+      <c r="L471">
+        <v>1</v>
+      </c>
+      <c r="M471">
+        <v>1</v>
+      </c>
+      <c r="N471">
+        <v>1</v>
+      </c>
+      <c r="Q471" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="472" spans="1:17">
+      <c r="A472">
+        <v>20</v>
+      </c>
+      <c r="B472">
+        <v>5</v>
+      </c>
+      <c r="C472">
+        <v>20280945</v>
+      </c>
+      <c r="D472" t="s">
+        <v>30</v>
+      </c>
+      <c r="E472">
+        <v>0.3113</v>
+      </c>
+      <c r="F472">
+        <v>-38.13662379287393</v>
+      </c>
+      <c r="G472">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H472">
+        <v>1.873939845609129E-05</v>
+      </c>
+      <c r="I472">
+        <v>5</v>
+      </c>
+      <c r="J472">
+        <v>1</v>
+      </c>
+      <c r="K472">
+        <v>0.5433070866141733</v>
+      </c>
+      <c r="L472">
+        <v>1</v>
+      </c>
+      <c r="M472">
+        <v>1</v>
+      </c>
+      <c r="N472">
+        <v>1</v>
+      </c>
+      <c r="Q472" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="473" spans="1:17">
+      <c r="A473">
+        <v>20</v>
+      </c>
+      <c r="B473">
+        <v>5</v>
+      </c>
+      <c r="C473">
+        <v>20280945</v>
+      </c>
+      <c r="D473" t="s">
+        <v>28</v>
+      </c>
+      <c r="E473">
+        <v>0.1022</v>
+      </c>
+      <c r="F473">
+        <v>-37.77204045954045</v>
+      </c>
+      <c r="G473">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H473">
+        <v>0.364602072731941</v>
+      </c>
+      <c r="I473">
+        <v>5</v>
+      </c>
+      <c r="J473">
+        <v>1</v>
+      </c>
+      <c r="K473">
+        <v>0.5275590551181102</v>
+      </c>
+      <c r="L473">
+        <v>1</v>
+      </c>
+      <c r="M473">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N473">
+        <v>1</v>
+      </c>
+      <c r="Q473" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="474" spans="1:17">
+      <c r="A474">
+        <v>20</v>
+      </c>
+      <c r="B474">
+        <v>5</v>
+      </c>
+      <c r="C474">
+        <v>20280945</v>
+      </c>
+      <c r="D474" t="s">
+        <v>27</v>
+      </c>
+      <c r="E474">
+        <v>0.3045</v>
+      </c>
+      <c r="F474">
+        <v>-38.13662379287393</v>
+      </c>
+      <c r="G474">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H474">
+        <v>1.873939845609129E-05</v>
+      </c>
+      <c r="I474">
+        <v>5</v>
+      </c>
+      <c r="J474">
+        <v>1</v>
+      </c>
+      <c r="K474">
+        <v>0.5433070866141733</v>
+      </c>
+      <c r="L474">
+        <v>1</v>
+      </c>
+      <c r="M474">
+        <v>1</v>
+      </c>
+      <c r="N474">
+        <v>1</v>
+      </c>
+      <c r="Q474" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="475" spans="1:17">
+      <c r="A475">
+        <v>20</v>
+      </c>
+      <c r="B475">
+        <v>5</v>
+      </c>
+      <c r="C475">
+        <v>20280945</v>
+      </c>
+      <c r="D475" t="s">
+        <v>29</v>
+      </c>
+      <c r="E475">
+        <v>206.1572</v>
+      </c>
+      <c r="F475">
+        <v>-35.31244796869805</v>
+      </c>
+      <c r="G475">
+        <v>-38.13664253227239</v>
+      </c>
+      <c r="H475">
+        <v>2.824194563574338</v>
+      </c>
+      <c r="I475">
+        <v>5</v>
+      </c>
+      <c r="J475">
+        <v>1</v>
+      </c>
+      <c r="K475">
+        <v>0.5433070866141733</v>
+      </c>
+      <c r="L475">
+        <v>1</v>
+      </c>
+      <c r="M475">
+        <v>1</v>
+      </c>
+      <c r="N475">
+        <v>1</v>
+      </c>
+      <c r="O475">
+        <v>1.147726760675572E-05</v>
+      </c>
+      <c r="P475">
+        <v>450</v>
+      </c>
+      <c r="Q475" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="476" spans="1:17">
+      <c r="A476">
+        <v>20</v>
+      </c>
+      <c r="B476">
+        <v>5</v>
+      </c>
+      <c r="C476">
+        <v>20280946</v>
+      </c>
+      <c r="D476" t="s">
+        <v>25</v>
+      </c>
+      <c r="E476">
+        <v>0.0003</v>
+      </c>
+      <c r="F476">
+        <v>-32.27892842451661</v>
+      </c>
+      <c r="G476">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H476">
+        <v>9.361985356383002</v>
+      </c>
+      <c r="I476">
+        <v>5</v>
+      </c>
+      <c r="J476">
+        <v>1</v>
+      </c>
+      <c r="K476">
+        <v>0.4626865671641791</v>
+      </c>
+      <c r="L476">
+        <v>1</v>
+      </c>
+      <c r="M476">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N476">
+        <v>1</v>
+      </c>
+      <c r="Q476" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="477" spans="1:17">
+      <c r="A477">
+        <v>20</v>
+      </c>
+      <c r="B477">
+        <v>5</v>
+      </c>
+      <c r="C477">
+        <v>20280946</v>
+      </c>
+      <c r="D477" t="s">
+        <v>26</v>
+      </c>
+      <c r="E477">
+        <v>0.0004</v>
+      </c>
+      <c r="F477">
+        <v>-37.23650418209229</v>
+      </c>
+      <c r="G477">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H477">
+        <v>4.40440959880732</v>
+      </c>
+      <c r="I477">
+        <v>5</v>
+      </c>
+      <c r="J477">
+        <v>1</v>
+      </c>
+      <c r="K477">
+        <v>0.5373134328358209</v>
+      </c>
+      <c r="L477">
+        <v>1</v>
+      </c>
+      <c r="M477">
+        <v>1</v>
+      </c>
+      <c r="N477">
+        <v>1</v>
+      </c>
+      <c r="Q477" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="478" spans="1:17">
+      <c r="A478">
+        <v>20</v>
+      </c>
+      <c r="B478">
+        <v>5</v>
+      </c>
+      <c r="C478">
+        <v>20280946</v>
+      </c>
+      <c r="D478" t="s">
+        <v>30</v>
+      </c>
+      <c r="E478">
+        <v>0.3114</v>
+      </c>
+      <c r="F478">
+        <v>-41.64091594679826</v>
+      </c>
+      <c r="G478">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H478">
+        <v>-2.165898649764131E-06</v>
+      </c>
+      <c r="I478">
+        <v>5</v>
+      </c>
+      <c r="J478">
+        <v>1</v>
+      </c>
+      <c r="K478">
+        <v>0.5223880597014925</v>
+      </c>
+      <c r="L478">
+        <v>1</v>
+      </c>
+      <c r="M478">
+        <v>1</v>
+      </c>
+      <c r="N478">
+        <v>1</v>
+      </c>
+      <c r="Q478" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="479" spans="1:17">
+      <c r="A479">
+        <v>20</v>
+      </c>
+      <c r="B479">
+        <v>5</v>
+      </c>
+      <c r="C479">
+        <v>20280946</v>
+      </c>
+      <c r="D479" t="s">
+        <v>28</v>
+      </c>
+      <c r="E479">
+        <v>0.0905</v>
+      </c>
+      <c r="F479">
+        <v>-40.59924928013152</v>
+      </c>
+      <c r="G479">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H479">
+        <v>1.041664500768093</v>
+      </c>
+      <c r="I479">
+        <v>5</v>
+      </c>
+      <c r="J479">
+        <v>1</v>
+      </c>
+      <c r="K479">
+        <v>0.5074626865671642</v>
+      </c>
+      <c r="L479">
+        <v>1</v>
+      </c>
+      <c r="M479">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N479">
+        <v>1</v>
+      </c>
+      <c r="Q479" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="480" spans="1:17">
+      <c r="A480">
+        <v>20</v>
+      </c>
+      <c r="B480">
+        <v>5</v>
+      </c>
+      <c r="C480">
+        <v>20280946</v>
+      </c>
+      <c r="D480" t="s">
+        <v>27</v>
+      </c>
+      <c r="E480">
+        <v>0.2811</v>
+      </c>
+      <c r="F480">
+        <v>-41.64091594679826</v>
+      </c>
+      <c r="G480">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H480">
+        <v>-2.165898649764131E-06</v>
+      </c>
+      <c r="I480">
+        <v>5</v>
+      </c>
+      <c r="J480">
+        <v>1</v>
+      </c>
+      <c r="K480">
+        <v>0.5223880597014925</v>
+      </c>
+      <c r="L480">
+        <v>1</v>
+      </c>
+      <c r="M480">
+        <v>1</v>
+      </c>
+      <c r="N480">
+        <v>1</v>
+      </c>
+      <c r="Q480" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="481" spans="1:17">
+      <c r="A481">
+        <v>20</v>
+      </c>
+      <c r="B481">
+        <v>5</v>
+      </c>
+      <c r="C481">
+        <v>20280946</v>
+      </c>
+      <c r="D481" t="s">
+        <v>29</v>
+      </c>
+      <c r="E481">
+        <v>329.575</v>
+      </c>
+      <c r="F481">
+        <v>-38.69938296997123</v>
+      </c>
+      <c r="G481">
+        <v>-41.64091378089961</v>
+      </c>
+      <c r="H481">
+        <v>2.941530810928384</v>
+      </c>
+      <c r="I481">
+        <v>5</v>
+      </c>
+      <c r="J481">
+        <v>1</v>
+      </c>
+      <c r="K481">
+        <v>0.5149253731343284</v>
+      </c>
+      <c r="L481">
+        <v>1</v>
+      </c>
+      <c r="M481">
+        <v>1</v>
+      </c>
+      <c r="N481">
+        <v>1</v>
+      </c>
+      <c r="O481">
+        <v>1.441360169409104E-05</v>
+      </c>
+      <c r="P481">
+        <v>450</v>
+      </c>
+      <c r="Q481" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="482" spans="1:17">
+      <c r="A482">
+        <v>20</v>
+      </c>
+      <c r="B482">
+        <v>5</v>
+      </c>
+      <c r="C482">
+        <v>20280947</v>
+      </c>
+      <c r="D482" t="s">
+        <v>25</v>
+      </c>
+      <c r="E482">
+        <v>0.0002</v>
+      </c>
+      <c r="F482">
+        <v>-19.13000749250739</v>
+      </c>
+      <c r="G482">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H482">
+        <v>15.65563330616612</v>
+      </c>
+      <c r="I482">
+        <v>5</v>
+      </c>
+      <c r="J482">
+        <v>1</v>
+      </c>
+      <c r="K482">
+        <v>0.4576271186440678</v>
+      </c>
+      <c r="L482">
+        <v>1</v>
+      </c>
+      <c r="M482">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N482">
+        <v>1</v>
+      </c>
+      <c r="Q482" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="483" spans="1:17">
+      <c r="A483">
+        <v>20</v>
+      </c>
+      <c r="B483">
+        <v>5</v>
+      </c>
+      <c r="C483">
+        <v>20280947</v>
+      </c>
+      <c r="D483" t="s">
+        <v>26</v>
+      </c>
+      <c r="E483">
+        <v>0.0004</v>
+      </c>
+      <c r="F483">
+        <v>-30.05596903096909</v>
+      </c>
+      <c r="G483">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H483">
+        <v>4.729671767704417</v>
+      </c>
+      <c r="I483">
+        <v>5</v>
+      </c>
+      <c r="J483">
+        <v>1</v>
+      </c>
+      <c r="K483">
+        <v>0.559322033898305</v>
+      </c>
+      <c r="L483">
+        <v>1</v>
+      </c>
+      <c r="M483">
+        <v>1</v>
+      </c>
+      <c r="N483">
+        <v>1</v>
+      </c>
+      <c r="Q483" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="484" spans="1:17">
+      <c r="A484">
+        <v>20</v>
+      </c>
+      <c r="B484">
+        <v>5</v>
+      </c>
+      <c r="C484">
+        <v>20280947</v>
+      </c>
+      <c r="D484" t="s">
+        <v>30</v>
+      </c>
+      <c r="E484">
+        <v>0.2766</v>
+      </c>
+      <c r="F484">
+        <v>-34.78562589371404</v>
+      </c>
+      <c r="G484">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H484">
+        <v>1.490495947109594E-05</v>
+      </c>
+      <c r="I484">
+        <v>5</v>
+      </c>
+      <c r="J484">
+        <v>1</v>
+      </c>
+      <c r="K484">
+        <v>0.5677966101694916</v>
+      </c>
+      <c r="L484">
+        <v>1</v>
+      </c>
+      <c r="M484">
+        <v>1</v>
+      </c>
+      <c r="N484">
+        <v>1</v>
+      </c>
+      <c r="Q484" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="485" spans="1:17">
+      <c r="A485">
+        <v>20</v>
+      </c>
+      <c r="B485">
+        <v>5</v>
+      </c>
+      <c r="C485">
+        <v>20280947</v>
+      </c>
+      <c r="D485" t="s">
+        <v>28</v>
+      </c>
+      <c r="E485">
+        <v>0.0522</v>
+      </c>
+      <c r="F485">
+        <v>-32.88562589371406</v>
+      </c>
+      <c r="G485">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H485">
+        <v>1.900014904959448</v>
+      </c>
+      <c r="I485">
+        <v>5</v>
+      </c>
+      <c r="J485">
+        <v>1</v>
+      </c>
+      <c r="K485">
+        <v>0.5677966101694916</v>
+      </c>
+      <c r="L485">
+        <v>1</v>
+      </c>
+      <c r="M485">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N485">
+        <v>1</v>
+      </c>
+      <c r="Q485" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="486" spans="1:17">
+      <c r="A486">
+        <v>20</v>
+      </c>
+      <c r="B486">
+        <v>5</v>
+      </c>
+      <c r="C486">
+        <v>20280947</v>
+      </c>
+      <c r="D486" t="s">
+        <v>27</v>
+      </c>
+      <c r="E486">
+        <v>0.3332</v>
+      </c>
+      <c r="F486">
+        <v>-34.78562589371404</v>
+      </c>
+      <c r="G486">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H486">
+        <v>1.490495947109594E-05</v>
+      </c>
+      <c r="I486">
+        <v>5</v>
+      </c>
+      <c r="J486">
+        <v>1</v>
+      </c>
+      <c r="K486">
+        <v>0.5677966101694916</v>
+      </c>
+      <c r="L486">
+        <v>1</v>
+      </c>
+      <c r="M486">
+        <v>1</v>
+      </c>
+      <c r="N486">
+        <v>1</v>
+      </c>
+      <c r="Q486" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="487" spans="1:17">
+      <c r="A487">
+        <v>20</v>
+      </c>
+      <c r="B487">
+        <v>5</v>
+      </c>
+      <c r="C487">
+        <v>20280947</v>
+      </c>
+      <c r="D487" t="s">
+        <v>29</v>
+      </c>
+      <c r="E487">
+        <v>205.0952</v>
+      </c>
+      <c r="F487">
+        <v>-32.58513569763568</v>
+      </c>
+      <c r="G487">
+        <v>-34.78564079867351</v>
+      </c>
+      <c r="H487">
+        <v>2.200505101037834</v>
+      </c>
+      <c r="I487">
+        <v>5</v>
+      </c>
+      <c r="J487">
+        <v>1</v>
+      </c>
+      <c r="K487">
+        <v>0.5423728813559322</v>
+      </c>
+      <c r="L487">
+        <v>1</v>
+      </c>
+      <c r="M487">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N487">
+        <v>1</v>
+      </c>
+      <c r="O487">
+        <v>1.509472611675305E-05</v>
+      </c>
+      <c r="P487">
+        <v>450</v>
+      </c>
+      <c r="Q487" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="488" spans="1:17">
+      <c r="A488">
+        <v>20</v>
+      </c>
+      <c r="B488">
+        <v>5</v>
+      </c>
+      <c r="C488">
+        <v>20280948</v>
+      </c>
+      <c r="D488" t="s">
+        <v>25</v>
+      </c>
+      <c r="E488">
+        <v>0.0002</v>
+      </c>
+      <c r="F488">
+        <v>-29.63977272727277</v>
+      </c>
+      <c r="G488">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H488">
+        <v>14.25033017113094</v>
+      </c>
+      <c r="I488">
+        <v>5</v>
+      </c>
+      <c r="J488">
+        <v>1</v>
+      </c>
+      <c r="K488">
+        <v>0.5038167938931297</v>
+      </c>
+      <c r="L488">
+        <v>1</v>
+      </c>
+      <c r="M488">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N488">
+        <v>1</v>
+      </c>
+      <c r="Q488" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="489" spans="1:17">
+      <c r="A489">
+        <v>20</v>
+      </c>
+      <c r="B489">
+        <v>5</v>
+      </c>
+      <c r="C489">
+        <v>20280948</v>
+      </c>
+      <c r="D489" t="s">
+        <v>26</v>
+      </c>
+      <c r="E489">
+        <v>0.0004</v>
+      </c>
+      <c r="F489">
+        <v>-40.55219155844157</v>
+      </c>
+      <c r="G489">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H489">
+        <v>3.337911339962147</v>
+      </c>
+      <c r="I489">
+        <v>5</v>
+      </c>
+      <c r="J489">
+        <v>1</v>
+      </c>
+      <c r="K489">
+        <v>0.5496183206106871</v>
+      </c>
+      <c r="L489">
+        <v>1</v>
+      </c>
+      <c r="M489">
+        <v>1</v>
+      </c>
+      <c r="N489">
+        <v>1</v>
+      </c>
+      <c r="Q489" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="490" spans="1:17">
+      <c r="A490">
+        <v>20</v>
+      </c>
+      <c r="B490">
+        <v>5</v>
+      </c>
+      <c r="C490">
+        <v>20280948</v>
+      </c>
+      <c r="D490" t="s">
+        <v>30</v>
+      </c>
+      <c r="E490">
+        <v>0.3264</v>
+      </c>
+      <c r="F490">
+        <v>-43.89007034632039</v>
+      </c>
+      <c r="G490">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H490">
+        <v>3.255208332575421E-05</v>
+      </c>
+      <c r="I490">
+        <v>5</v>
+      </c>
+      <c r="J490">
+        <v>1</v>
+      </c>
+      <c r="K490">
+        <v>0.5190839694656488</v>
+      </c>
+      <c r="L490">
+        <v>1</v>
+      </c>
+      <c r="M490">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N490">
+        <v>1</v>
+      </c>
+      <c r="Q490" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="491" spans="1:17">
+      <c r="A491">
+        <v>20</v>
+      </c>
+      <c r="B491">
+        <v>5</v>
+      </c>
+      <c r="C491">
+        <v>20280948</v>
+      </c>
+      <c r="D491" t="s">
+        <v>28</v>
+      </c>
+      <c r="E491">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="F491">
+        <v>-42.55673701298701</v>
+      </c>
+      <c r="G491">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H491">
+        <v>1.333365885416697</v>
+      </c>
+      <c r="I491">
+        <v>5</v>
+      </c>
+      <c r="J491">
+        <v>1</v>
+      </c>
+      <c r="K491">
+        <v>0.4961832061068702</v>
+      </c>
+      <c r="L491">
+        <v>1</v>
+      </c>
+      <c r="M491">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N491">
+        <v>1</v>
+      </c>
+      <c r="Q491" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="492" spans="1:17">
+      <c r="A492">
+        <v>20</v>
+      </c>
+      <c r="B492">
+        <v>5</v>
+      </c>
+      <c r="C492">
+        <v>20280948</v>
+      </c>
+      <c r="D492" t="s">
+        <v>27</v>
+      </c>
+      <c r="E492">
+        <v>0.3281</v>
+      </c>
+      <c r="F492">
+        <v>-43.89007034632039</v>
+      </c>
+      <c r="G492">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H492">
+        <v>3.255208332575421E-05</v>
+      </c>
+      <c r="I492">
+        <v>5</v>
+      </c>
+      <c r="J492">
+        <v>1</v>
+      </c>
+      <c r="K492">
+        <v>0.5190839694656488</v>
+      </c>
+      <c r="L492">
+        <v>1</v>
+      </c>
+      <c r="M492">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N492">
+        <v>1</v>
+      </c>
+      <c r="Q492" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="493" spans="1:17">
+      <c r="A493">
+        <v>20</v>
+      </c>
+      <c r="B493">
+        <v>5</v>
+      </c>
+      <c r="C493">
+        <v>20280948</v>
+      </c>
+      <c r="D493" t="s">
+        <v>29</v>
+      </c>
+      <c r="E493">
+        <v>202.5145</v>
+      </c>
+      <c r="F493">
+        <v>-42.81128246753269</v>
+      </c>
+      <c r="G493">
+        <v>-43.89010289840371</v>
+      </c>
+      <c r="H493">
+        <v>1.078820430871019</v>
+      </c>
+      <c r="I493">
+        <v>5</v>
+      </c>
+      <c r="J493">
+        <v>1</v>
+      </c>
+      <c r="K493">
+        <v>0.5114503816793893</v>
+      </c>
+      <c r="L493">
+        <v>1</v>
+      </c>
+      <c r="M493">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N493">
+        <v>1</v>
+      </c>
+      <c r="O493">
+        <v>1.32810066727928E-05</v>
+      </c>
+      <c r="P493">
+        <v>450</v>
+      </c>
+      <c r="Q493" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="494" spans="1:17">
+      <c r="A494">
+        <v>20</v>
+      </c>
+      <c r="B494">
+        <v>5</v>
+      </c>
+      <c r="C494">
+        <v>20280949</v>
+      </c>
+      <c r="D494" t="s">
+        <v>25</v>
+      </c>
+      <c r="E494">
+        <v>0.0002</v>
+      </c>
+      <c r="F494">
+        <v>-28.40449452508278</v>
+      </c>
+      <c r="G494">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H494">
+        <v>14.72103977732786</v>
+      </c>
+      <c r="I494">
+        <v>5</v>
+      </c>
+      <c r="J494">
+        <v>1</v>
+      </c>
+      <c r="K494">
+        <v>0.4651162790697674</v>
+      </c>
+      <c r="L494">
+        <v>0.875</v>
+      </c>
+      <c r="M494">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N494">
+        <v>1</v>
+      </c>
+      <c r="Q494" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="495" spans="1:17">
+      <c r="A495">
+        <v>20</v>
+      </c>
+      <c r="B495">
+        <v>5</v>
+      </c>
+      <c r="C495">
+        <v>20280949</v>
+      </c>
+      <c r="D495" t="s">
+        <v>26</v>
+      </c>
+      <c r="E495">
+        <v>0.0003</v>
+      </c>
+      <c r="F495">
+        <v>-40.73390628978859</v>
+      </c>
+      <c r="G495">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H495">
+        <v>2.39162801262205</v>
+      </c>
+      <c r="I495">
+        <v>5</v>
+      </c>
+      <c r="J495">
+        <v>1</v>
+      </c>
+      <c r="K495">
+        <v>0.5581395348837209</v>
+      </c>
+      <c r="L495">
+        <v>1</v>
+      </c>
+      <c r="M495">
+        <v>1</v>
+      </c>
+      <c r="N495">
+        <v>1</v>
+      </c>
+      <c r="Q495" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="496" spans="1:17">
+      <c r="A496">
+        <v>20</v>
+      </c>
+      <c r="B496">
+        <v>5</v>
+      </c>
+      <c r="C496">
+        <v>20280949</v>
+      </c>
+      <c r="D496" t="s">
+        <v>30</v>
+      </c>
+      <c r="E496">
+        <v>0.2701</v>
+      </c>
+      <c r="F496">
+        <v>-43.12557295645536</v>
+      </c>
+      <c r="G496">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H496">
+        <v>-3.865404471525835E-05</v>
+      </c>
+      <c r="I496">
+        <v>5</v>
+      </c>
+      <c r="J496">
+        <v>1</v>
+      </c>
+      <c r="K496">
+        <v>0.5581395348837209</v>
+      </c>
+      <c r="L496">
+        <v>1</v>
+      </c>
+      <c r="M496">
+        <v>1</v>
+      </c>
+      <c r="N496">
+        <v>1</v>
+      </c>
+      <c r="Q496" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="497" spans="1:17">
+      <c r="A497">
+        <v>20</v>
+      </c>
+      <c r="B497">
+        <v>5</v>
+      </c>
+      <c r="C497">
+        <v>20280949</v>
+      </c>
+      <c r="D497" t="s">
+        <v>28</v>
+      </c>
+      <c r="E497">
+        <v>0.08260000000000001</v>
+      </c>
+      <c r="F497">
+        <v>-41.45057295645529</v>
+      </c>
+      <c r="G497">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H497">
+        <v>1.674961345955353</v>
+      </c>
+      <c r="I497">
+        <v>5</v>
+      </c>
+      <c r="J497">
+        <v>1</v>
+      </c>
+      <c r="K497">
+        <v>0.5581395348837209</v>
+      </c>
+      <c r="L497">
+        <v>1</v>
+      </c>
+      <c r="M497">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N497">
+        <v>1</v>
+      </c>
+      <c r="Q497" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="498" spans="1:17">
+      <c r="A498">
+        <v>20</v>
+      </c>
+      <c r="B498">
+        <v>5</v>
+      </c>
+      <c r="C498">
+        <v>20280949</v>
+      </c>
+      <c r="D498" t="s">
+        <v>27</v>
+      </c>
+      <c r="E498">
+        <v>0.3394</v>
+      </c>
+      <c r="F498">
+        <v>-43.12557295645536</v>
+      </c>
+      <c r="G498">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H498">
+        <v>-3.865404471525835E-05</v>
+      </c>
+      <c r="I498">
+        <v>5</v>
+      </c>
+      <c r="J498">
+        <v>1</v>
+      </c>
+      <c r="K498">
+        <v>0.5581395348837209</v>
+      </c>
+      <c r="L498">
+        <v>1</v>
+      </c>
+      <c r="M498">
+        <v>1</v>
+      </c>
+      <c r="N498">
+        <v>1</v>
+      </c>
+      <c r="Q498" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="499" spans="1:17">
+      <c r="A499">
+        <v>20</v>
+      </c>
+      <c r="B499">
+        <v>5</v>
+      </c>
+      <c r="C499">
+        <v>20280949</v>
+      </c>
+      <c r="D499" t="s">
+        <v>29</v>
+      </c>
+      <c r="E499">
+        <v>205.7117</v>
+      </c>
+      <c r="F499">
+        <v>-38.91953781512598</v>
+      </c>
+      <c r="G499">
+        <v>-43.12553430241064</v>
+      </c>
+      <c r="H499">
+        <v>4.205996487284665</v>
+      </c>
+      <c r="I499">
+        <v>5</v>
+      </c>
+      <c r="J499">
+        <v>1</v>
+      </c>
+      <c r="K499">
+        <v>0.5271317829457365</v>
+      </c>
+      <c r="L499">
+        <v>1</v>
+      </c>
+      <c r="M499">
+        <v>1</v>
+      </c>
+      <c r="N499">
+        <v>1</v>
+      </c>
+      <c r="O499">
+        <v>1.950582216342924E-05</v>
+      </c>
+      <c r="P499">
+        <v>450</v>
+      </c>
+      <c r="Q499" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="500" spans="1:17">
+      <c r="A500">
+        <v>20</v>
+      </c>
+      <c r="B500">
+        <v>5</v>
+      </c>
+      <c r="C500">
+        <v>20280950</v>
+      </c>
+      <c r="D500" t="s">
+        <v>25</v>
+      </c>
+      <c r="E500">
+        <v>0.0002</v>
+      </c>
+      <c r="F500">
+        <v>-26.67979104229107</v>
+      </c>
+      <c r="G500">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H500">
+        <v>12.97173004404453</v>
+      </c>
+      <c r="I500">
+        <v>5</v>
+      </c>
+      <c r="J500">
+        <v>1</v>
+      </c>
+      <c r="K500">
+        <v>0.4761904761904761</v>
+      </c>
+      <c r="L500">
+        <v>1</v>
+      </c>
+      <c r="M500">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N500">
+        <v>1</v>
+      </c>
+      <c r="Q500" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="501" spans="1:17">
+      <c r="A501">
+        <v>20</v>
+      </c>
+      <c r="B501">
+        <v>5</v>
+      </c>
+      <c r="C501">
+        <v>20280950</v>
+      </c>
+      <c r="D501" t="s">
+        <v>26</v>
+      </c>
+      <c r="E501">
+        <v>0.0003</v>
+      </c>
+      <c r="F501">
+        <v>-38.72301448551434</v>
+      </c>
+      <c r="G501">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H501">
+        <v>0.9285066008212652</v>
+      </c>
+      <c r="I501">
+        <v>5</v>
+      </c>
+      <c r="J501">
+        <v>1</v>
+      </c>
+      <c r="K501">
+        <v>0.5634920634920635</v>
+      </c>
+      <c r="L501">
+        <v>1</v>
+      </c>
+      <c r="M501">
+        <v>1</v>
+      </c>
+      <c r="N501">
+        <v>1</v>
+      </c>
+      <c r="Q501" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="502" spans="1:17">
+      <c r="A502">
+        <v>20</v>
+      </c>
+      <c r="B502">
+        <v>5</v>
+      </c>
+      <c r="C502">
+        <v>20280950</v>
+      </c>
+      <c r="D502" t="s">
+        <v>30</v>
+      </c>
+      <c r="E502">
+        <v>0.275</v>
+      </c>
+      <c r="F502">
+        <v>-39.6515859140859</v>
+      </c>
+      <c r="G502">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H502">
+        <v>-6.482775029326149E-05</v>
+      </c>
+      <c r="I502">
+        <v>5</v>
+      </c>
+      <c r="J502">
+        <v>1</v>
+      </c>
+      <c r="K502">
+        <v>0.5396825396825397</v>
+      </c>
+      <c r="L502">
+        <v>1</v>
+      </c>
+      <c r="M502">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N502">
+        <v>1</v>
+      </c>
+      <c r="Q502" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="503" spans="1:17">
+      <c r="A503">
+        <v>20</v>
+      </c>
+      <c r="B503">
+        <v>5</v>
+      </c>
+      <c r="C503">
+        <v>20280950</v>
+      </c>
+      <c r="D503" t="s">
+        <v>28</v>
+      </c>
+      <c r="E503">
+        <v>2.5467</v>
+      </c>
+      <c r="F503">
+        <v>-39.03491924741934</v>
+      </c>
+      <c r="G503">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H503">
+        <v>0.6166018389162673</v>
+      </c>
+      <c r="I503">
+        <v>5</v>
+      </c>
+      <c r="J503">
+        <v>1</v>
+      </c>
+      <c r="K503">
+        <v>0.5317460317460317</v>
+      </c>
+      <c r="L503">
+        <v>1</v>
+      </c>
+      <c r="M503">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N503">
+        <v>1</v>
+      </c>
+      <c r="Q503" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="504" spans="1:17">
+      <c r="A504">
+        <v>20</v>
+      </c>
+      <c r="B504">
+        <v>5</v>
+      </c>
+      <c r="C504">
+        <v>20280950</v>
+      </c>
+      <c r="D504" t="s">
+        <v>27</v>
+      </c>
+      <c r="E504">
+        <v>0.5773</v>
+      </c>
+      <c r="F504">
+        <v>-39.6515859140859</v>
+      </c>
+      <c r="G504">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H504">
+        <v>-6.482775029326149E-05</v>
+      </c>
+      <c r="I504">
+        <v>5</v>
+      </c>
+      <c r="J504">
+        <v>1</v>
+      </c>
+      <c r="K504">
+        <v>0.5396825396825397</v>
+      </c>
+      <c r="L504">
+        <v>1</v>
+      </c>
+      <c r="M504">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N504">
+        <v>1</v>
+      </c>
+      <c r="Q504" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="505" spans="1:17">
+      <c r="A505">
+        <v>20</v>
+      </c>
+      <c r="B505">
+        <v>5</v>
+      </c>
+      <c r="C505">
+        <v>20280950</v>
+      </c>
+      <c r="D505" t="s">
+        <v>29</v>
+      </c>
+      <c r="E505">
+        <v>209.7549</v>
+      </c>
+      <c r="F505">
+        <v>-36.98275474525474</v>
+      </c>
+      <c r="G505">
+        <v>-39.65152108633561</v>
+      </c>
+      <c r="H505">
+        <v>2.668766341080868</v>
+      </c>
+      <c r="I505">
+        <v>5</v>
+      </c>
+      <c r="J505">
+        <v>1</v>
+      </c>
+      <c r="K505">
+        <v>0.5238095238095238</v>
+      </c>
+      <c r="L505">
+        <v>1</v>
+      </c>
+      <c r="M505">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N505">
+        <v>1</v>
+      </c>
+      <c r="O505">
+        <v>1.486135534047812E-05</v>
+      </c>
+      <c r="P505">
+        <v>450</v>
+      </c>
+      <c r="Q505" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="506" spans="1:17">
+      <c r="A506">
+        <v>20</v>
+      </c>
+      <c r="B506">
+        <v>5</v>
+      </c>
+      <c r="C506">
+        <v>20280951</v>
+      </c>
+      <c r="D506" t="s">
+        <v>25</v>
+      </c>
+      <c r="E506">
+        <v>0.0003</v>
+      </c>
+      <c r="F506">
+        <v>-32.91228673287492</v>
+      </c>
+      <c r="G506">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H506">
+        <v>4.469875409325596</v>
+      </c>
+      <c r="I506">
+        <v>5</v>
+      </c>
+      <c r="J506">
+        <v>1</v>
+      </c>
+      <c r="K506">
+        <v>0.5327868852459017</v>
+      </c>
+      <c r="L506">
+        <v>1</v>
+      </c>
+      <c r="M506">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N506">
+        <v>1</v>
+      </c>
+      <c r="Q506" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="507" spans="1:17">
+      <c r="A507">
+        <v>20</v>
+      </c>
+      <c r="B507">
+        <v>5</v>
+      </c>
+      <c r="C507">
+        <v>20280951</v>
+      </c>
+      <c r="D507" t="s">
+        <v>26</v>
+      </c>
+      <c r="E507">
+        <v>0.0003</v>
+      </c>
+      <c r="F507">
+        <v>-35.00774127832949</v>
+      </c>
+      <c r="G507">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H507">
+        <v>2.374420863871024</v>
+      </c>
+      <c r="I507">
+        <v>5</v>
+      </c>
+      <c r="J507">
+        <v>1</v>
+      </c>
+      <c r="K507">
+        <v>0.5901639344262295</v>
+      </c>
+      <c r="L507">
+        <v>1</v>
+      </c>
+      <c r="M507">
+        <v>1</v>
+      </c>
+      <c r="N507">
+        <v>1</v>
+      </c>
+      <c r="Q507" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="508" spans="1:17">
+      <c r="A508">
+        <v>20</v>
+      </c>
+      <c r="B508">
+        <v>5</v>
+      </c>
+      <c r="C508">
+        <v>20280951</v>
+      </c>
+      <c r="D508" t="s">
+        <v>30</v>
+      </c>
+      <c r="E508">
+        <v>0.252</v>
+      </c>
+      <c r="F508">
+        <v>-37.38217468805692</v>
+      </c>
+      <c r="G508">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H508">
+        <v>-1.254585640708683E-05</v>
+      </c>
+      <c r="I508">
+        <v>5</v>
+      </c>
+      <c r="J508">
+        <v>1</v>
+      </c>
+      <c r="K508">
+        <v>0.5245901639344263</v>
+      </c>
+      <c r="L508">
+        <v>1</v>
+      </c>
+      <c r="M508">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N508">
+        <v>1</v>
+      </c>
+      <c r="Q508" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="509" spans="1:17">
+      <c r="A509">
+        <v>20</v>
+      </c>
+      <c r="B509">
+        <v>5</v>
+      </c>
+      <c r="C509">
+        <v>20280951</v>
+      </c>
+      <c r="D509" t="s">
+        <v>28</v>
+      </c>
+      <c r="E509">
+        <v>0.0905</v>
+      </c>
+      <c r="F509">
+        <v>-36.25381970970204</v>
+      </c>
+      <c r="G509">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H509">
+        <v>1.128342432498471</v>
+      </c>
+      <c r="I509">
+        <v>5</v>
+      </c>
+      <c r="J509">
+        <v>1</v>
+      </c>
+      <c r="K509">
+        <v>0.5491803278688525</v>
+      </c>
+      <c r="L509">
+        <v>1</v>
+      </c>
+      <c r="M509">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N509">
+        <v>1</v>
+      </c>
+      <c r="Q509" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="510" spans="1:17">
+      <c r="A510">
+        <v>20</v>
+      </c>
+      <c r="B510">
+        <v>5</v>
+      </c>
+      <c r="C510">
+        <v>20280951</v>
+      </c>
+      <c r="D510" t="s">
+        <v>27</v>
+      </c>
+      <c r="E510">
+        <v>0.3138</v>
+      </c>
+      <c r="F510">
+        <v>-37.38217468805692</v>
+      </c>
+      <c r="G510">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H510">
+        <v>-1.254585640708683E-05</v>
+      </c>
+      <c r="I510">
+        <v>5</v>
+      </c>
+      <c r="J510">
+        <v>1</v>
+      </c>
+      <c r="K510">
+        <v>0.5245901639344263</v>
+      </c>
+      <c r="L510">
+        <v>1</v>
+      </c>
+      <c r="M510">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N510">
+        <v>1</v>
+      </c>
+      <c r="Q510" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="511" spans="1:17">
+      <c r="A511">
+        <v>20</v>
+      </c>
+      <c r="B511">
+        <v>5</v>
+      </c>
+      <c r="C511">
+        <v>20280951</v>
+      </c>
+      <c r="D511" t="s">
+        <v>29</v>
+      </c>
+      <c r="E511">
+        <v>202.4817</v>
+      </c>
+      <c r="F511">
+        <v>-34.70262923351152</v>
+      </c>
+      <c r="G511">
+        <v>-37.38216214220051</v>
+      </c>
+      <c r="H511">
+        <v>2.679532908688998</v>
+      </c>
+      <c r="I511">
+        <v>5</v>
+      </c>
+      <c r="J511">
+        <v>1</v>
+      </c>
+      <c r="K511">
+        <v>0.5245901639344263</v>
+      </c>
+      <c r="L511">
+        <v>1</v>
+      </c>
+      <c r="M511">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N511">
+        <v>1</v>
+      </c>
+      <c r="O511">
+        <v>1.638064412312262E-05</v>
+      </c>
+      <c r="P511">
+        <v>450</v>
+      </c>
+      <c r="Q511" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="512" spans="1:17">
+      <c r="A512">
+        <v>20</v>
+      </c>
+      <c r="B512">
+        <v>5</v>
+      </c>
+      <c r="C512">
+        <v>20280952</v>
+      </c>
+      <c r="D512" t="s">
+        <v>25</v>
+      </c>
+      <c r="E512">
+        <v>0.0003</v>
+      </c>
+      <c r="F512">
+        <v>-27.82527472527477</v>
+      </c>
+      <c r="G512">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H512">
+        <v>13.0539758256067</v>
+      </c>
+      <c r="I512">
+        <v>5</v>
+      </c>
+      <c r="J512">
+        <v>1</v>
+      </c>
+      <c r="K512">
+        <v>0.4436090225563909</v>
+      </c>
+      <c r="L512">
+        <v>1</v>
+      </c>
+      <c r="M512">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="N512">
+        <v>1</v>
+      </c>
+      <c r="Q512" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="513" spans="1:17">
+      <c r="A513">
+        <v>20</v>
+      </c>
+      <c r="B513">
+        <v>5</v>
+      </c>
+      <c r="C513">
+        <v>20280952</v>
+      </c>
+      <c r="D513" t="s">
+        <v>26</v>
+      </c>
+      <c r="E513">
+        <v>0.0004</v>
+      </c>
+      <c r="F513">
+        <v>-32.10540293040287</v>
+      </c>
+      <c r="G513">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H513">
+        <v>8.773847620478591</v>
+      </c>
+      <c r="I513">
+        <v>5</v>
+      </c>
+      <c r="J513">
+        <v>1</v>
+      </c>
+      <c r="K513">
+        <v>0.5112781954887218</v>
+      </c>
+      <c r="L513">
+        <v>1</v>
+      </c>
+      <c r="M513">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N513">
+        <v>1</v>
+      </c>
+      <c r="Q513" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="514" spans="1:17">
+      <c r="A514">
+        <v>20</v>
+      </c>
+      <c r="B514">
+        <v>5</v>
+      </c>
+      <c r="C514">
+        <v>20280952</v>
+      </c>
+      <c r="D514" t="s">
+        <v>30</v>
+      </c>
+      <c r="E514">
+        <v>0.28</v>
+      </c>
+      <c r="F514">
+        <v>-40.87921245421239</v>
+      </c>
+      <c r="G514">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H514">
+        <v>3.809666907272913E-05</v>
+      </c>
+      <c r="I514">
+        <v>5</v>
+      </c>
+      <c r="J514">
+        <v>1</v>
+      </c>
+      <c r="K514">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="L514">
+        <v>1</v>
+      </c>
+      <c r="M514">
+        <v>1</v>
+      </c>
+      <c r="N514">
+        <v>1</v>
+      </c>
+      <c r="Q514" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="515" spans="1:17">
+      <c r="A515">
+        <v>20</v>
+      </c>
+      <c r="B515">
+        <v>5</v>
+      </c>
+      <c r="C515">
+        <v>20280952</v>
+      </c>
+      <c r="D515" t="s">
+        <v>28</v>
+      </c>
+      <c r="E515">
+        <v>0.0756</v>
+      </c>
+      <c r="F515">
+        <v>-40.47170329670337</v>
+      </c>
+      <c r="G515">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H515">
+        <v>0.4075472541780982</v>
+      </c>
+      <c r="I515">
+        <v>5</v>
+      </c>
+      <c r="J515">
+        <v>1</v>
+      </c>
+      <c r="K515">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="L515">
+        <v>1</v>
+      </c>
+      <c r="M515">
+        <v>1</v>
+      </c>
+      <c r="N515">
+        <v>1</v>
+      </c>
+      <c r="Q515" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="516" spans="1:17">
+      <c r="A516">
+        <v>20</v>
+      </c>
+      <c r="B516">
+        <v>5</v>
+      </c>
+      <c r="C516">
+        <v>20280952</v>
+      </c>
+      <c r="D516" t="s">
+        <v>27</v>
+      </c>
+      <c r="E516">
+        <v>0.3064</v>
+      </c>
+      <c r="F516">
+        <v>-40.87921245421239</v>
+      </c>
+      <c r="G516">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H516">
+        <v>3.809666907272913E-05</v>
+      </c>
+      <c r="I516">
+        <v>5</v>
+      </c>
+      <c r="J516">
+        <v>1</v>
+      </c>
+      <c r="K516">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="L516">
+        <v>1</v>
+      </c>
+      <c r="M516">
+        <v>1</v>
+      </c>
+      <c r="N516">
+        <v>1</v>
+      </c>
+      <c r="Q516" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="517" spans="1:17">
+      <c r="A517">
+        <v>20</v>
+      </c>
+      <c r="B517">
+        <v>5</v>
+      </c>
+      <c r="C517">
+        <v>20280952</v>
+      </c>
+      <c r="D517" t="s">
+        <v>29</v>
+      </c>
+      <c r="E517">
+        <v>208.8598</v>
+      </c>
+      <c r="F517">
+        <v>-38.96254578754576</v>
+      </c>
+      <c r="G517">
+        <v>-40.87925055088147</v>
+      </c>
+      <c r="H517">
+        <v>1.916704763335701</v>
+      </c>
+      <c r="I517">
+        <v>5</v>
+      </c>
+      <c r="J517">
+        <v>1</v>
+      </c>
+      <c r="K517">
+        <v>0.518796992481203</v>
+      </c>
+      <c r="L517">
+        <v>1</v>
+      </c>
+      <c r="M517">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N517">
+        <v>1</v>
+      </c>
+      <c r="O517">
+        <v>1.713038442639665E-05</v>
+      </c>
+      <c r="P517">
+        <v>450</v>
+      </c>
+      <c r="Q517" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="518" spans="1:17">
+      <c r="A518">
+        <v>20</v>
+      </c>
+      <c r="B518">
+        <v>5</v>
+      </c>
+      <c r="C518">
+        <v>20280953</v>
+      </c>
+      <c r="D518" t="s">
+        <v>25</v>
+      </c>
+      <c r="E518">
+        <v>0.0016</v>
+      </c>
+      <c r="F518">
+        <v>-24.0100815850816</v>
+      </c>
+      <c r="G518">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H518">
+        <v>18.46779090457073</v>
+      </c>
+      <c r="I518">
+        <v>5</v>
+      </c>
+      <c r="J518">
+        <v>1</v>
+      </c>
+      <c r="K518">
+        <v>0.453125</v>
+      </c>
+      <c r="L518">
+        <v>1</v>
+      </c>
+      <c r="M518">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N518">
+        <v>1</v>
+      </c>
+      <c r="Q518" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="519" spans="1:17">
+      <c r="A519">
+        <v>20</v>
+      </c>
+      <c r="B519">
+        <v>5</v>
+      </c>
+      <c r="C519">
+        <v>20280953</v>
+      </c>
+      <c r="D519" t="s">
+        <v>26</v>
+      </c>
+      <c r="E519">
+        <v>0.0009</v>
+      </c>
+      <c r="F519">
+        <v>-37.78856143856149</v>
+      </c>
+      <c r="G519">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H519">
+        <v>4.68931105109084</v>
+      </c>
+      <c r="I519">
+        <v>5</v>
+      </c>
+      <c r="J519">
+        <v>1</v>
+      </c>
+      <c r="K519">
+        <v>0.5625</v>
+      </c>
+      <c r="L519">
+        <v>1</v>
+      </c>
+      <c r="M519">
+        <v>1</v>
+      </c>
+      <c r="N519">
+        <v>1</v>
+      </c>
+      <c r="Q519" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="520" spans="1:17">
+      <c r="A520">
+        <v>20</v>
+      </c>
+      <c r="B520">
+        <v>5</v>
+      </c>
+      <c r="C520">
+        <v>20280953</v>
+      </c>
+      <c r="D520" t="s">
+        <v>30</v>
+      </c>
+      <c r="E520">
+        <v>0.3697</v>
+      </c>
+      <c r="F520">
+        <v>-42.47784715284718</v>
+      </c>
+      <c r="G520">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H520">
+        <v>2.533680515171E-05</v>
+      </c>
+      <c r="I520">
+        <v>5</v>
+      </c>
+      <c r="J520">
+        <v>1</v>
+      </c>
+      <c r="K520">
+        <v>0.53125</v>
+      </c>
+      <c r="L520">
+        <v>1</v>
+      </c>
+      <c r="M520">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N520">
+        <v>0.8</v>
+      </c>
+      <c r="Q520" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="521" spans="1:17">
+      <c r="A521">
+        <v>20</v>
+      </c>
+      <c r="B521">
+        <v>5</v>
+      </c>
+      <c r="C521">
+        <v>20280953</v>
+      </c>
+      <c r="D521" t="s">
+        <v>28</v>
+      </c>
+      <c r="E521">
+        <v>0.102</v>
+      </c>
+      <c r="F521">
+        <v>-39.60284715284729</v>
+      </c>
+      <c r="G521">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H521">
+        <v>2.875025336805038</v>
+      </c>
+      <c r="I521">
+        <v>5</v>
+      </c>
+      <c r="J521">
+        <v>1</v>
+      </c>
+      <c r="K521">
+        <v>0.53125</v>
+      </c>
+      <c r="L521">
+        <v>1</v>
+      </c>
+      <c r="M521">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N521">
+        <v>0.8</v>
+      </c>
+      <c r="Q521" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="522" spans="1:17">
+      <c r="A522">
+        <v>20</v>
+      </c>
+      <c r="B522">
+        <v>5</v>
+      </c>
+      <c r="C522">
+        <v>20280953</v>
+      </c>
+      <c r="D522" t="s">
+        <v>27</v>
+      </c>
+      <c r="E522">
+        <v>0.3304</v>
+      </c>
+      <c r="F522">
+        <v>-42.47784715284718</v>
+      </c>
+      <c r="G522">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H522">
+        <v>2.533680515171E-05</v>
+      </c>
+      <c r="I522">
+        <v>5</v>
+      </c>
+      <c r="J522">
+        <v>1</v>
+      </c>
+      <c r="K522">
+        <v>0.53125</v>
+      </c>
+      <c r="L522">
+        <v>1</v>
+      </c>
+      <c r="M522">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N522">
+        <v>0.8</v>
+      </c>
+      <c r="Q522" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="523" spans="1:17">
+      <c r="A523">
+        <v>20</v>
+      </c>
+      <c r="B523">
+        <v>5</v>
+      </c>
+      <c r="C523">
+        <v>20280953</v>
+      </c>
+      <c r="D523" t="s">
+        <v>29</v>
+      </c>
+      <c r="E523">
+        <v>330.6168</v>
+      </c>
+      <c r="F523">
+        <v>-40.63477355977364</v>
+      </c>
+      <c r="G523">
+        <v>-42.47787248965233</v>
+      </c>
+      <c r="H523">
+        <v>1.843098929878693</v>
+      </c>
+      <c r="I523">
+        <v>5</v>
+      </c>
+      <c r="J523">
+        <v>1</v>
+      </c>
+      <c r="K523">
+        <v>0.515625</v>
+      </c>
+      <c r="L523">
+        <v>1</v>
+      </c>
+      <c r="M523">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N523">
+        <v>0.8</v>
+      </c>
+      <c r="O523">
+        <v>1.456588200321149E-05</v>
+      </c>
+      <c r="P523">
+        <v>450</v>
+      </c>
+      <c r="Q523" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="524" spans="1:17">
+      <c r="A524">
+        <v>20</v>
+      </c>
+      <c r="B524">
+        <v>5</v>
+      </c>
+      <c r="C524">
+        <v>20280954</v>
+      </c>
+      <c r="D524" t="s">
+        <v>25</v>
+      </c>
+      <c r="E524">
+        <v>0.0002</v>
+      </c>
+      <c r="F524">
+        <v>-32.99026390276401</v>
+      </c>
+      <c r="G524">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H524">
+        <v>10.11288892585264</v>
+      </c>
+      <c r="I524">
+        <v>5</v>
+      </c>
+      <c r="J524">
+        <v>1</v>
+      </c>
+      <c r="K524">
+        <v>0.4571428571428571</v>
+      </c>
+      <c r="L524">
+        <v>1</v>
+      </c>
+      <c r="M524">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N524">
+        <v>1</v>
+      </c>
+      <c r="Q524" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="525" spans="1:17">
+      <c r="A525">
+        <v>20</v>
+      </c>
+      <c r="B525">
+        <v>5</v>
+      </c>
+      <c r="C525">
+        <v>20280954</v>
+      </c>
+      <c r="D525" t="s">
+        <v>26</v>
+      </c>
+      <c r="E525">
+        <v>0.0003</v>
+      </c>
+      <c r="F525">
+        <v>-34.60081793206803</v>
+      </c>
+      <c r="G525">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H525">
+        <v>8.502334896548632</v>
+      </c>
+      <c r="I525">
+        <v>5</v>
+      </c>
+      <c r="J525">
+        <v>1</v>
+      </c>
+      <c r="K525">
+        <v>0.5071428571428571</v>
+      </c>
+      <c r="L525">
+        <v>1</v>
+      </c>
+      <c r="M525">
+        <v>1</v>
+      </c>
+      <c r="N525">
+        <v>1</v>
+      </c>
+      <c r="Q525" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="526" spans="1:17">
+      <c r="A526">
+        <v>20</v>
+      </c>
+      <c r="B526">
+        <v>5</v>
+      </c>
+      <c r="C526">
+        <v>20280954</v>
+      </c>
+      <c r="D526" t="s">
+        <v>30</v>
+      </c>
+      <c r="E526">
+        <v>0.2799</v>
+      </c>
+      <c r="F526">
+        <v>-43.10319888444906</v>
+      </c>
+      <c r="G526">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H526">
+        <v>-4.605583239936095E-05</v>
+      </c>
+      <c r="I526">
+        <v>5</v>
+      </c>
+      <c r="J526">
+        <v>1</v>
+      </c>
+      <c r="K526">
+        <v>0.5</v>
+      </c>
+      <c r="L526">
+        <v>1</v>
+      </c>
+      <c r="M526">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N526">
+        <v>1</v>
+      </c>
+      <c r="Q526" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="527" spans="1:17">
+      <c r="A527">
+        <v>20</v>
+      </c>
+      <c r="B527">
+        <v>5</v>
+      </c>
+      <c r="C527">
+        <v>20280954</v>
+      </c>
+      <c r="D527" t="s">
+        <v>28</v>
+      </c>
+      <c r="E527">
+        <v>0.0757</v>
+      </c>
+      <c r="F527">
+        <v>-42.21986555111562</v>
+      </c>
+      <c r="G527">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H527">
+        <v>0.8832872775010401</v>
+      </c>
+      <c r="I527">
+        <v>5</v>
+      </c>
+      <c r="J527">
+        <v>1</v>
+      </c>
+      <c r="K527">
+        <v>0.4928571428571429</v>
+      </c>
+      <c r="L527">
+        <v>1</v>
+      </c>
+      <c r="M527">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N527">
+        <v>1</v>
+      </c>
+      <c r="Q527" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="528" spans="1:17">
+      <c r="A528">
+        <v>20</v>
+      </c>
+      <c r="B528">
+        <v>5</v>
+      </c>
+      <c r="C528">
+        <v>20280954</v>
+      </c>
+      <c r="D528" t="s">
+        <v>27</v>
+      </c>
+      <c r="E528">
+        <v>0.3508</v>
+      </c>
+      <c r="F528">
+        <v>-43.10319888444906</v>
+      </c>
+      <c r="G528">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H528">
+        <v>-4.605583239936095E-05</v>
+      </c>
+      <c r="I528">
+        <v>5</v>
+      </c>
+      <c r="J528">
+        <v>1</v>
+      </c>
+      <c r="K528">
+        <v>0.5</v>
+      </c>
+      <c r="L528">
+        <v>1</v>
+      </c>
+      <c r="M528">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N528">
+        <v>1</v>
+      </c>
+      <c r="Q528" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="529" spans="1:17">
+      <c r="A529">
+        <v>20</v>
+      </c>
+      <c r="B529">
+        <v>5</v>
+      </c>
+      <c r="C529">
+        <v>20280954</v>
+      </c>
+      <c r="D529" t="s">
+        <v>29</v>
+      </c>
+      <c r="E529">
+        <v>209.5652</v>
+      </c>
+      <c r="F529">
+        <v>-40.73565184815186</v>
+      </c>
+      <c r="G529">
+        <v>-43.10315282861666</v>
+      </c>
+      <c r="H529">
+        <v>2.367500980464797</v>
+      </c>
+      <c r="I529">
+        <v>5</v>
+      </c>
+      <c r="J529">
+        <v>1</v>
+      </c>
+      <c r="K529">
+        <v>0.5071428571428571</v>
+      </c>
+      <c r="L529">
+        <v>1</v>
+      </c>
+      <c r="M529">
+        <v>1</v>
+      </c>
+      <c r="N529">
+        <v>1</v>
+      </c>
+      <c r="O529">
+        <v>1.626639102350275E-05</v>
+      </c>
+      <c r="P529">
+        <v>450</v>
+      </c>
+      <c r="Q529" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="530" spans="1:17">
+      <c r="A530">
+        <v>20</v>
+      </c>
+      <c r="B530">
+        <v>5</v>
+      </c>
+      <c r="C530">
+        <v>20280955</v>
+      </c>
+      <c r="D530" t="s">
+        <v>25</v>
+      </c>
+      <c r="E530">
+        <v>0.0002</v>
+      </c>
+      <c r="F530">
+        <v>-36.52803030303028</v>
+      </c>
+      <c r="G530">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H530">
+        <v>5.543557912356732</v>
+      </c>
+      <c r="I530">
+        <v>5</v>
+      </c>
+      <c r="J530">
+        <v>1</v>
+      </c>
+      <c r="K530">
+        <v>0.4927536231884058</v>
+      </c>
+      <c r="L530">
+        <v>1</v>
+      </c>
+      <c r="M530">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N530">
+        <v>1</v>
+      </c>
+      <c r="Q530" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="531" spans="1:17">
+      <c r="A531">
+        <v>20</v>
+      </c>
+      <c r="B531">
+        <v>5</v>
+      </c>
+      <c r="C531">
+        <v>20280955</v>
+      </c>
+      <c r="D531" t="s">
+        <v>26</v>
+      </c>
+      <c r="E531">
+        <v>0.0003</v>
+      </c>
+      <c r="F531">
+        <v>-37.85495337995349</v>
+      </c>
+      <c r="G531">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H531">
+        <v>4.216634835433524</v>
+      </c>
+      <c r="I531">
+        <v>5</v>
+      </c>
+      <c r="J531">
+        <v>1</v>
+      </c>
+      <c r="K531">
+        <v>0.5144927536231884</v>
+      </c>
+      <c r="L531">
+        <v>1</v>
+      </c>
+      <c r="M531">
+        <v>1</v>
+      </c>
+      <c r="N531">
+        <v>1</v>
+      </c>
+      <c r="Q531" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="532" spans="1:17">
+      <c r="A532">
+        <v>20</v>
+      </c>
+      <c r="B532">
+        <v>5</v>
+      </c>
+      <c r="C532">
+        <v>20280955</v>
+      </c>
+      <c r="D532" t="s">
+        <v>30</v>
+      </c>
+      <c r="E532">
+        <v>0.2664</v>
+      </c>
+      <c r="F532">
+        <v>-42.07162004662007</v>
+      </c>
+      <c r="G532">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H532">
+        <v>-3.183123305916524E-05</v>
+      </c>
+      <c r="I532">
+        <v>5</v>
+      </c>
+      <c r="J532">
+        <v>1</v>
+      </c>
+      <c r="K532">
+        <v>0.5144927536231884</v>
+      </c>
+      <c r="L532">
+        <v>1</v>
+      </c>
+      <c r="M532">
+        <v>1</v>
+      </c>
+      <c r="N532">
+        <v>1</v>
+      </c>
+      <c r="Q532" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="533" spans="1:17">
+      <c r="A533">
+        <v>20</v>
+      </c>
+      <c r="B533">
+        <v>5</v>
+      </c>
+      <c r="C533">
+        <v>20280955</v>
+      </c>
+      <c r="D533" t="s">
+        <v>28</v>
+      </c>
+      <c r="E533">
+        <v>0.0842</v>
+      </c>
+      <c r="F533">
+        <v>-40.72439782439801</v>
+      </c>
+      <c r="G533">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H533">
+        <v>1.347190390988999</v>
+      </c>
+      <c r="I533">
+        <v>5</v>
+      </c>
+      <c r="J533">
+        <v>1</v>
+      </c>
+      <c r="K533">
+        <v>0.5289855072463768</v>
+      </c>
+      <c r="L533">
+        <v>1</v>
+      </c>
+      <c r="M533">
+        <v>1</v>
+      </c>
+      <c r="N533">
+        <v>1</v>
+      </c>
+      <c r="Q533" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="534" spans="1:17">
+      <c r="A534">
+        <v>20</v>
+      </c>
+      <c r="B534">
+        <v>5</v>
+      </c>
+      <c r="C534">
+        <v>20280955</v>
+      </c>
+      <c r="D534" t="s">
+        <v>27</v>
+      </c>
+      <c r="E534">
+        <v>0.2709</v>
+      </c>
+      <c r="F534">
+        <v>-42.07162004662007</v>
+      </c>
+      <c r="G534">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H534">
+        <v>-3.183123305916524E-05</v>
+      </c>
+      <c r="I534">
+        <v>5</v>
+      </c>
+      <c r="J534">
+        <v>1</v>
+      </c>
+      <c r="K534">
+        <v>0.5144927536231884</v>
+      </c>
+      <c r="L534">
+        <v>1</v>
+      </c>
+      <c r="M534">
+        <v>1</v>
+      </c>
+      <c r="N534">
+        <v>1</v>
+      </c>
+      <c r="Q534" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="535" spans="1:17">
+      <c r="A535">
+        <v>20</v>
+      </c>
+      <c r="B535">
+        <v>5</v>
+      </c>
+      <c r="C535">
+        <v>20280955</v>
+      </c>
+      <c r="D535" t="s">
+        <v>29</v>
+      </c>
+      <c r="E535">
+        <v>205.0771</v>
+      </c>
+      <c r="F535">
+        <v>-40.35174825174829</v>
+      </c>
+      <c r="G535">
+        <v>-42.07158821538701</v>
+      </c>
+      <c r="H535">
+        <v>1.719839963638719</v>
+      </c>
+      <c r="I535">
+        <v>5</v>
+      </c>
+      <c r="J535">
+        <v>1</v>
+      </c>
+      <c r="K535">
+        <v>0.5144927536231884</v>
+      </c>
+      <c r="L535">
+        <v>1</v>
+      </c>
+      <c r="M535">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N535">
+        <v>1</v>
+      </c>
+      <c r="O535">
+        <v>1.710879636505888E-05</v>
+      </c>
+      <c r="P535">
+        <v>450</v>
+      </c>
+      <c r="Q535" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="536" spans="1:17">
+      <c r="A536">
+        <v>20</v>
+      </c>
+      <c r="B536">
+        <v>5</v>
+      </c>
+      <c r="C536">
+        <v>20280956</v>
+      </c>
+      <c r="D536" t="s">
+        <v>25</v>
+      </c>
+      <c r="E536">
+        <v>0.0002</v>
+      </c>
+      <c r="F536">
+        <v>-32.32142857142856</v>
+      </c>
+      <c r="G536">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H536">
+        <v>8.965426974826414</v>
+      </c>
+      <c r="I536">
+        <v>5</v>
+      </c>
+      <c r="J536">
+        <v>1</v>
+      </c>
+      <c r="K536">
+        <v>0.4883720930232558</v>
+      </c>
+      <c r="L536">
+        <v>1</v>
+      </c>
+      <c r="M536">
+        <v>0.9230769230769232</v>
+      </c>
+      <c r="N536">
+        <v>1</v>
+      </c>
+      <c r="Q536" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="537" spans="1:17">
+      <c r="A537">
+        <v>20</v>
+      </c>
+      <c r="B537">
+        <v>5</v>
+      </c>
+      <c r="C537">
+        <v>20280956</v>
+      </c>
+      <c r="D537" t="s">
+        <v>26</v>
+      </c>
+      <c r="E537">
+        <v>0.0003</v>
+      </c>
+      <c r="F537">
+        <v>-37.64097985347985</v>
+      </c>
+      <c r="G537">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H537">
+        <v>3.645875692775121</v>
+      </c>
+      <c r="I537">
+        <v>5</v>
+      </c>
+      <c r="J537">
+        <v>1</v>
+      </c>
+      <c r="K537">
+        <v>0.5426356589147286</v>
+      </c>
+      <c r="L537">
+        <v>1</v>
+      </c>
+      <c r="M537">
+        <v>1</v>
+      </c>
+      <c r="N537">
+        <v>1</v>
+      </c>
+      <c r="Q537" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="538" spans="1:17">
+      <c r="A538">
+        <v>20</v>
+      </c>
+      <c r="B538">
+        <v>5</v>
+      </c>
+      <c r="C538">
+        <v>20280956</v>
+      </c>
+      <c r="D538" t="s">
+        <v>30</v>
+      </c>
+      <c r="E538">
+        <v>0.2312</v>
+      </c>
+      <c r="F538">
+        <v>-41.28681318681311</v>
+      </c>
+      <c r="G538">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H538">
+        <v>4.235944186348206E-05</v>
+      </c>
+      <c r="I538">
+        <v>5</v>
+      </c>
+      <c r="J538">
+        <v>1</v>
+      </c>
+      <c r="K538">
+        <v>0.5503875968992248</v>
+      </c>
+      <c r="L538">
+        <v>1</v>
+      </c>
+      <c r="M538">
+        <v>1</v>
+      </c>
+      <c r="N538">
+        <v>1</v>
+      </c>
+      <c r="Q538" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="539" spans="1:17">
+      <c r="A539">
+        <v>20</v>
+      </c>
+      <c r="B539">
+        <v>5</v>
+      </c>
+      <c r="C539">
+        <v>20280956</v>
+      </c>
+      <c r="D539" t="s">
+        <v>28</v>
+      </c>
+      <c r="E539">
+        <v>0.07580000000000001</v>
+      </c>
+      <c r="F539">
+        <v>-41.28681318681311</v>
+      </c>
+      <c r="G539">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H539">
+        <v>4.235944186348206E-05</v>
+      </c>
+      <c r="I539">
+        <v>5</v>
+      </c>
+      <c r="J539">
+        <v>1</v>
+      </c>
+      <c r="K539">
+        <v>0.5503875968992248</v>
+      </c>
+      <c r="L539">
+        <v>1</v>
+      </c>
+      <c r="M539">
+        <v>1</v>
+      </c>
+      <c r="N539">
+        <v>1</v>
+      </c>
+      <c r="Q539" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="540" spans="1:17">
+      <c r="A540">
+        <v>20</v>
+      </c>
+      <c r="B540">
+        <v>5</v>
+      </c>
+      <c r="C540">
+        <v>20280956</v>
+      </c>
+      <c r="D540" t="s">
+        <v>27</v>
+      </c>
+      <c r="E540">
+        <v>0.3504</v>
+      </c>
+      <c r="F540">
+        <v>-41.28681318681311</v>
+      </c>
+      <c r="G540">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H540">
+        <v>4.235944186348206E-05</v>
+      </c>
+      <c r="I540">
+        <v>5</v>
+      </c>
+      <c r="J540">
+        <v>1</v>
+      </c>
+      <c r="K540">
+        <v>0.5503875968992248</v>
+      </c>
+      <c r="L540">
+        <v>1</v>
+      </c>
+      <c r="M540">
+        <v>1</v>
+      </c>
+      <c r="N540">
+        <v>1</v>
+      </c>
+      <c r="Q540" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="541" spans="1:17">
+      <c r="A541">
+        <v>20</v>
+      </c>
+      <c r="B541">
+        <v>5</v>
+      </c>
+      <c r="C541">
+        <v>20280956</v>
+      </c>
+      <c r="D541" t="s">
+        <v>29</v>
+      </c>
+      <c r="E541">
+        <v>204.4169</v>
+      </c>
+      <c r="F541">
+        <v>-37.90883699633707</v>
+      </c>
+      <c r="G541">
+        <v>-41.28685554625497</v>
+      </c>
+      <c r="H541">
+        <v>3.378018549917897</v>
+      </c>
+      <c r="I541">
+        <v>5</v>
+      </c>
+      <c r="J541">
+        <v>1</v>
+      </c>
+      <c r="K541">
+        <v>0.5193798449612403</v>
+      </c>
+      <c r="L541">
+        <v>1</v>
+      </c>
+      <c r="M541">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N541">
+        <v>1</v>
+      </c>
+      <c r="O541">
+        <v>1.591958512429766E-05</v>
+      </c>
+      <c r="P541">
+        <v>450</v>
+      </c>
+      <c r="Q541" t="s">
+        <v>218</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>